<commit_message>
demo: updated data forms
</commit_message>
<xml_diff>
--- a/Demo/lf-integrated/demo_lf_itas_9999_2_part.xlsx
+++ b/Demo/lf-integrated/demo_lf_itas_9999_2_part.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\lf-integrated\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97F804BA-39FB-4B21-B6B0-04732801F0B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{479F1601-B4D6-4F40-BDC3-C91DEE2854AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -624,9 +624,6 @@
     <t>${p_site_id}</t>
   </si>
   <si>
-    <t>${p_index_init} + indexed-repeat(${position}, ${p9999}, count(${p9999}))</t>
-  </si>
-  <si>
     <t>Profession</t>
   </si>
   <si>
@@ -636,10 +633,13 @@
     <t>demo_lf_itas_9999_2_part</t>
   </si>
   <si>
-    <t>pi9999</t>
-  </si>
-  <si>
     <t>(Demo) 2. ITAS LF-ONCHO LF Participant From</t>
+  </si>
+  <si>
+    <t>pi999</t>
+  </si>
+  <si>
+    <t>${p_index_init} + indexed-repeat(${position}, ${pi999}, count(${pi999}))</t>
   </si>
 </sst>
 </file>
@@ -1550,7 +1550,7 @@
       <c r="G11" s="10"/>
       <c r="H11" s="10"/>
       <c r="I11" s="10" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="J11" s="10"/>
       <c r="K11" s="10"/>
@@ -2240,7 +2240,7 @@
         <v>176</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H42" s="7" t="s">
         <v>82</v>
@@ -2487,7 +2487,7 @@
         <v>102</v>
       </c>
       <c r="I57" s="10" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="J57" s="10"/>
       <c r="K57" s="10"/>
@@ -2812,10 +2812,10 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="7" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C2" t="s">
         <v>48</v>

</xml_diff>